<commit_message>
Controller archive read: SAU array and InteliMains register maps from the Neo's own definitions, archive reader tool, configuration write-up, history findings
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Modbus_Register_Map_Rev.1.0.xlsx
+++ b/docs/turkey/Solar_Modbus_Register_Map_Rev.1.0.xlsx
@@ -1182,6 +1182,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>1010</v>
       </c>
@@ -2308,6 +2309,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
         <v>1039</v>
       </c>
@@ -3434,6 +3436,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="n">
         <v>1068</v>
       </c>
@@ -4560,6 +4563,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="n">
         <v>1097</v>
       </c>
@@ -5686,6 +5690,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F128" t="inlineStr"/>
       <c r="G128" t="n">
         <v>1126</v>
       </c>
@@ -6812,6 +6817,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F157" t="inlineStr"/>
       <c r="G157" t="n">
         <v>1155</v>
       </c>
@@ -7938,6 +7944,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F186" t="inlineStr"/>
       <c r="G186" t="n">
         <v>1184</v>
       </c>
@@ -9064,6 +9071,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F215" t="inlineStr"/>
       <c r="G215" t="n">
         <v>1213</v>
       </c>
@@ -10190,6 +10198,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F244" t="inlineStr"/>
       <c r="G244" t="n">
         <v>1242</v>
       </c>
@@ -11316,6 +11325,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F273" t="inlineStr"/>
       <c r="G273" t="n">
         <v>1271</v>
       </c>
@@ -12257,12 +12267,12 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>pv-meter.energy_delivered_kwh</t>
-        </is>
-      </c>
-      <c r="I297" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+          <t>pv-array.energy_total_kwh</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -12481,6 +12491,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F303" t="inlineStr"/>
       <c r="G303" t="n">
         <v>1301</v>
       </c>
@@ -12515,6 +12526,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F304" t="inlineStr"/>
       <c r="G304" t="n">
         <v>1302</v>
       </c>
@@ -12549,6 +12561,7 @@
           <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
+      <c r="F305" t="inlineStr"/>
       <c r="G305" t="n">
         <v>1303</v>
       </c>
@@ -12593,12 +12606,12 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>pv-meter.energy_total_kwh</t>
-        </is>
-      </c>
-      <c r="I306" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+          <t>pv-array.energy_total_kwh</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inverters and PV array mapped from Sineng's TCP protocol document: unit ids 3-12, inverter registers, PV array addresses; Turkey map 300 of 305 tags ready
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Modbus_Register_Map_Rev.1.0.xlsx
+++ b/docs/turkey/Solar_Modbus_Register_Map_Rev.1.0.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>to be provided once the connection method (VPN) is agreed</t>
+          <t>to be provided with the test date (an address on the plant network, reserved with the plant team)</t>
         </is>
       </c>
     </row>
@@ -805,9 +805,9 @@
           <t>inv-01.ac_power_kw</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -844,9 +844,9 @@
           <t>inv-01.current_l1_a</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -883,9 +883,9 @@
           <t>inv-01.current_l2_a</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -922,9 +922,9 @@
           <t>inv-01.current_l3_a</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -961,9 +961,9 @@
           <t>inv-01.dc_power_kw</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1000,9 +1000,9 @@
           <t>inv-01.frequency_hz</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1039,9 +1039,9 @@
           <t>inv-01.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1078,9 +1078,9 @@
           <t>inv-01.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1117,9 +1117,9 @@
           <t>inv-01.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1156,9 +1156,9 @@
           <t>inv-01.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1191,9 +1191,9 @@
           <t>inv-01.comm_error</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1230,9 +1230,9 @@
           <t>inv-01.string_current_1_a</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1269,9 +1269,9 @@
           <t>inv-01.string_current_2_a</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1308,9 +1308,9 @@
           <t>inv-01.string_current_3_a</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1347,9 +1347,9 @@
           <t>inv-01.string_current_4_a</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1386,9 +1386,9 @@
           <t>inv-01.string_current_5_a</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1425,9 +1425,9 @@
           <t>inv-01.string_current_6_a</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1464,9 +1464,9 @@
           <t>inv-01.string_current_7_a</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1503,9 +1503,9 @@
           <t>inv-01.string_current_8_a</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1542,9 +1542,9 @@
           <t>inv-01.string_current_9_a</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1581,9 +1581,9 @@
           <t>inv-01.string_current_10_a</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1620,9 +1620,9 @@
           <t>inv-01.string_current_11_a</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1659,9 +1659,9 @@
           <t>inv-01.string_current_12_a</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1698,9 +1698,9 @@
           <t>inv-01.string_current_13_a</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1737,9 +1737,9 @@
           <t>inv-01.string_current_14_a</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1776,9 +1776,9 @@
           <t>inv-01.string_current_15_a</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1815,9 +1815,9 @@
           <t>inv-01.string_current_16_a</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1854,9 +1854,9 @@
           <t>inv-01.string_current_17_a</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1893,9 +1893,9 @@
           <t>inv-01.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1932,9 +1932,9 @@
           <t>inv-02.ac_power_kw</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -1971,9 +1971,9 @@
           <t>inv-02.current_l1_a</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2010,9 +2010,9 @@
           <t>inv-02.current_l2_a</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2049,9 +2049,9 @@
           <t>inv-02.current_l3_a</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2088,9 +2088,9 @@
           <t>inv-02.dc_power_kw</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2127,9 +2127,9 @@
           <t>inv-02.frequency_hz</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2166,9 +2166,9 @@
           <t>inv-02.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2205,9 +2205,9 @@
           <t>inv-02.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2244,9 +2244,9 @@
           <t>inv-02.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2283,9 +2283,9 @@
           <t>inv-02.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2318,9 +2318,9 @@
           <t>inv-02.comm_error</t>
         </is>
       </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2357,9 +2357,9 @@
           <t>inv-02.string_current_1_a</t>
         </is>
       </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2396,9 +2396,9 @@
           <t>inv-02.string_current_2_a</t>
         </is>
       </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2435,9 +2435,9 @@
           <t>inv-02.string_current_3_a</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2474,9 +2474,9 @@
           <t>inv-02.string_current_4_a</t>
         </is>
       </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2513,9 +2513,9 @@
           <t>inv-02.string_current_5_a</t>
         </is>
       </c>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2552,9 +2552,9 @@
           <t>inv-02.string_current_6_a</t>
         </is>
       </c>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2591,9 +2591,9 @@
           <t>inv-02.string_current_7_a</t>
         </is>
       </c>
-      <c r="I48" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2630,9 +2630,9 @@
           <t>inv-02.string_current_8_a</t>
         </is>
       </c>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2669,9 +2669,9 @@
           <t>inv-02.string_current_9_a</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2708,9 +2708,9 @@
           <t>inv-02.string_current_10_a</t>
         </is>
       </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2747,9 +2747,9 @@
           <t>inv-02.string_current_11_a</t>
         </is>
       </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2786,9 +2786,9 @@
           <t>inv-02.string_current_12_a</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2825,9 +2825,9 @@
           <t>inv-02.string_current_13_a</t>
         </is>
       </c>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2864,9 +2864,9 @@
           <t>inv-02.string_current_14_a</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2903,9 +2903,9 @@
           <t>inv-02.string_current_15_a</t>
         </is>
       </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2942,9 +2942,9 @@
           <t>inv-02.string_current_16_a</t>
         </is>
       </c>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -2981,9 +2981,9 @@
           <t>inv-02.string_current_17_a</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3020,9 +3020,9 @@
           <t>inv-02.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3059,9 +3059,9 @@
           <t>inv-03.ac_power_kw</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3098,9 +3098,9 @@
           <t>inv-03.current_l1_a</t>
         </is>
       </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3137,9 +3137,9 @@
           <t>inv-03.current_l2_a</t>
         </is>
       </c>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3176,9 +3176,9 @@
           <t>inv-03.current_l3_a</t>
         </is>
       </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3215,9 +3215,9 @@
           <t>inv-03.dc_power_kw</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3254,9 +3254,9 @@
           <t>inv-03.frequency_hz</t>
         </is>
       </c>
-      <c r="I65" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3293,9 +3293,9 @@
           <t>inv-03.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3332,9 +3332,9 @@
           <t>inv-03.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I67" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3371,9 +3371,9 @@
           <t>inv-03.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3410,9 +3410,9 @@
           <t>inv-03.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3445,9 +3445,9 @@
           <t>inv-03.comm_error</t>
         </is>
       </c>
-      <c r="I70" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3484,9 +3484,9 @@
           <t>inv-03.string_current_1_a</t>
         </is>
       </c>
-      <c r="I71" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3523,9 +3523,9 @@
           <t>inv-03.string_current_2_a</t>
         </is>
       </c>
-      <c r="I72" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3562,9 +3562,9 @@
           <t>inv-03.string_current_3_a</t>
         </is>
       </c>
-      <c r="I73" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3601,9 +3601,9 @@
           <t>inv-03.string_current_4_a</t>
         </is>
       </c>
-      <c r="I74" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3640,9 +3640,9 @@
           <t>inv-03.string_current_5_a</t>
         </is>
       </c>
-      <c r="I75" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3679,9 +3679,9 @@
           <t>inv-03.string_current_6_a</t>
         </is>
       </c>
-      <c r="I76" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3718,9 +3718,9 @@
           <t>inv-03.string_current_7_a</t>
         </is>
       </c>
-      <c r="I77" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3757,9 +3757,9 @@
           <t>inv-03.string_current_8_a</t>
         </is>
       </c>
-      <c r="I78" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3796,9 +3796,9 @@
           <t>inv-03.string_current_9_a</t>
         </is>
       </c>
-      <c r="I79" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3835,9 +3835,9 @@
           <t>inv-03.string_current_10_a</t>
         </is>
       </c>
-      <c r="I80" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3874,9 +3874,9 @@
           <t>inv-03.string_current_11_a</t>
         </is>
       </c>
-      <c r="I81" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3913,9 +3913,9 @@
           <t>inv-03.string_current_12_a</t>
         </is>
       </c>
-      <c r="I82" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3952,9 +3952,9 @@
           <t>inv-03.string_current_13_a</t>
         </is>
       </c>
-      <c r="I83" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -3991,9 +3991,9 @@
           <t>inv-03.string_current_14_a</t>
         </is>
       </c>
-      <c r="I84" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4030,9 +4030,9 @@
           <t>inv-03.string_current_15_a</t>
         </is>
       </c>
-      <c r="I85" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4069,9 +4069,9 @@
           <t>inv-03.string_current_16_a</t>
         </is>
       </c>
-      <c r="I86" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4108,9 +4108,9 @@
           <t>inv-03.string_current_17_a</t>
         </is>
       </c>
-      <c r="I87" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4147,9 +4147,9 @@
           <t>inv-03.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I88" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4186,9 +4186,9 @@
           <t>inv-04.ac_power_kw</t>
         </is>
       </c>
-      <c r="I89" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4225,9 +4225,9 @@
           <t>inv-04.current_l1_a</t>
         </is>
       </c>
-      <c r="I90" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4264,9 +4264,9 @@
           <t>inv-04.current_l2_a</t>
         </is>
       </c>
-      <c r="I91" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4303,9 +4303,9 @@
           <t>inv-04.current_l3_a</t>
         </is>
       </c>
-      <c r="I92" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4342,9 +4342,9 @@
           <t>inv-04.dc_power_kw</t>
         </is>
       </c>
-      <c r="I93" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4381,9 +4381,9 @@
           <t>inv-04.frequency_hz</t>
         </is>
       </c>
-      <c r="I94" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4420,9 +4420,9 @@
           <t>inv-04.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I95" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4459,9 +4459,9 @@
           <t>inv-04.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I96" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4498,9 +4498,9 @@
           <t>inv-04.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I97" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4537,9 +4537,9 @@
           <t>inv-04.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I98" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4572,9 +4572,9 @@
           <t>inv-04.comm_error</t>
         </is>
       </c>
-      <c r="I99" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4611,9 +4611,9 @@
           <t>inv-04.string_current_1_a</t>
         </is>
       </c>
-      <c r="I100" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4650,9 +4650,9 @@
           <t>inv-04.string_current_2_a</t>
         </is>
       </c>
-      <c r="I101" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4689,9 +4689,9 @@
           <t>inv-04.string_current_3_a</t>
         </is>
       </c>
-      <c r="I102" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4728,9 +4728,9 @@
           <t>inv-04.string_current_4_a</t>
         </is>
       </c>
-      <c r="I103" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4767,9 +4767,9 @@
           <t>inv-04.string_current_5_a</t>
         </is>
       </c>
-      <c r="I104" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4806,9 +4806,9 @@
           <t>inv-04.string_current_6_a</t>
         </is>
       </c>
-      <c r="I105" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4845,9 +4845,9 @@
           <t>inv-04.string_current_7_a</t>
         </is>
       </c>
-      <c r="I106" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4884,9 +4884,9 @@
           <t>inv-04.string_current_8_a</t>
         </is>
       </c>
-      <c r="I107" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4923,9 +4923,9 @@
           <t>inv-04.string_current_9_a</t>
         </is>
       </c>
-      <c r="I108" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -4962,9 +4962,9 @@
           <t>inv-04.string_current_10_a</t>
         </is>
       </c>
-      <c r="I109" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5001,9 +5001,9 @@
           <t>inv-04.string_current_11_a</t>
         </is>
       </c>
-      <c r="I110" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5040,9 +5040,9 @@
           <t>inv-04.string_current_12_a</t>
         </is>
       </c>
-      <c r="I111" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5079,9 +5079,9 @@
           <t>inv-04.string_current_13_a</t>
         </is>
       </c>
-      <c r="I112" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5118,9 +5118,9 @@
           <t>inv-04.string_current_14_a</t>
         </is>
       </c>
-      <c r="I113" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5157,9 +5157,9 @@
           <t>inv-04.string_current_15_a</t>
         </is>
       </c>
-      <c r="I114" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5196,9 +5196,9 @@
           <t>inv-04.string_current_16_a</t>
         </is>
       </c>
-      <c r="I115" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5235,9 +5235,9 @@
           <t>inv-04.string_current_17_a</t>
         </is>
       </c>
-      <c r="I116" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5274,9 +5274,9 @@
           <t>inv-04.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I117" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5313,9 +5313,9 @@
           <t>inv-05.ac_power_kw</t>
         </is>
       </c>
-      <c r="I118" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5352,9 +5352,9 @@
           <t>inv-05.current_l1_a</t>
         </is>
       </c>
-      <c r="I119" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5391,9 +5391,9 @@
           <t>inv-05.current_l2_a</t>
         </is>
       </c>
-      <c r="I120" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5430,9 +5430,9 @@
           <t>inv-05.current_l3_a</t>
         </is>
       </c>
-      <c r="I121" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5469,9 +5469,9 @@
           <t>inv-05.dc_power_kw</t>
         </is>
       </c>
-      <c r="I122" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5508,9 +5508,9 @@
           <t>inv-05.frequency_hz</t>
         </is>
       </c>
-      <c r="I123" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5547,9 +5547,9 @@
           <t>inv-05.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I124" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5586,9 +5586,9 @@
           <t>inv-05.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I125" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5625,9 +5625,9 @@
           <t>inv-05.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I126" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5664,9 +5664,9 @@
           <t>inv-05.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I127" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5699,9 +5699,9 @@
           <t>inv-05.comm_error</t>
         </is>
       </c>
-      <c r="I128" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5738,9 +5738,9 @@
           <t>inv-05.string_current_1_a</t>
         </is>
       </c>
-      <c r="I129" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5777,9 +5777,9 @@
           <t>inv-05.string_current_2_a</t>
         </is>
       </c>
-      <c r="I130" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5816,9 +5816,9 @@
           <t>inv-05.string_current_3_a</t>
         </is>
       </c>
-      <c r="I131" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5855,9 +5855,9 @@
           <t>inv-05.string_current_4_a</t>
         </is>
       </c>
-      <c r="I132" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5894,9 +5894,9 @@
           <t>inv-05.string_current_5_a</t>
         </is>
       </c>
-      <c r="I133" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5933,9 +5933,9 @@
           <t>inv-05.string_current_6_a</t>
         </is>
       </c>
-      <c r="I134" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -5972,9 +5972,9 @@
           <t>inv-05.string_current_7_a</t>
         </is>
       </c>
-      <c r="I135" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6011,9 +6011,9 @@
           <t>inv-05.string_current_8_a</t>
         </is>
       </c>
-      <c r="I136" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6050,9 +6050,9 @@
           <t>inv-05.string_current_9_a</t>
         </is>
       </c>
-      <c r="I137" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6089,9 +6089,9 @@
           <t>inv-05.string_current_10_a</t>
         </is>
       </c>
-      <c r="I138" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6128,9 +6128,9 @@
           <t>inv-05.string_current_11_a</t>
         </is>
       </c>
-      <c r="I139" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6167,9 +6167,9 @@
           <t>inv-05.string_current_12_a</t>
         </is>
       </c>
-      <c r="I140" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6206,9 +6206,9 @@
           <t>inv-05.string_current_13_a</t>
         </is>
       </c>
-      <c r="I141" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6245,9 +6245,9 @@
           <t>inv-05.string_current_14_a</t>
         </is>
       </c>
-      <c r="I142" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6284,9 +6284,9 @@
           <t>inv-05.string_current_15_a</t>
         </is>
       </c>
-      <c r="I143" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6323,9 +6323,9 @@
           <t>inv-05.string_current_16_a</t>
         </is>
       </c>
-      <c r="I144" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6362,9 +6362,9 @@
           <t>inv-05.string_current_17_a</t>
         </is>
       </c>
-      <c r="I145" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6401,9 +6401,9 @@
           <t>inv-05.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I146" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6440,9 +6440,9 @@
           <t>inv-06.ac_power_kw</t>
         </is>
       </c>
-      <c r="I147" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6479,9 +6479,9 @@
           <t>inv-06.current_l1_a</t>
         </is>
       </c>
-      <c r="I148" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6518,9 +6518,9 @@
           <t>inv-06.current_l2_a</t>
         </is>
       </c>
-      <c r="I149" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6557,9 +6557,9 @@
           <t>inv-06.current_l3_a</t>
         </is>
       </c>
-      <c r="I150" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6596,9 +6596,9 @@
           <t>inv-06.dc_power_kw</t>
         </is>
       </c>
-      <c r="I151" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6635,9 +6635,9 @@
           <t>inv-06.frequency_hz</t>
         </is>
       </c>
-      <c r="I152" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6674,9 +6674,9 @@
           <t>inv-06.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I153" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6713,9 +6713,9 @@
           <t>inv-06.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I154" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6752,9 +6752,9 @@
           <t>inv-06.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I155" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6791,9 +6791,9 @@
           <t>inv-06.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I156" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6826,9 +6826,9 @@
           <t>inv-06.comm_error</t>
         </is>
       </c>
-      <c r="I157" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6865,9 +6865,9 @@
           <t>inv-06.string_current_1_a</t>
         </is>
       </c>
-      <c r="I158" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6904,9 +6904,9 @@
           <t>inv-06.string_current_2_a</t>
         </is>
       </c>
-      <c r="I159" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6943,9 +6943,9 @@
           <t>inv-06.string_current_3_a</t>
         </is>
       </c>
-      <c r="I160" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -6982,9 +6982,9 @@
           <t>inv-06.string_current_4_a</t>
         </is>
       </c>
-      <c r="I161" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7021,9 +7021,9 @@
           <t>inv-06.string_current_5_a</t>
         </is>
       </c>
-      <c r="I162" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7060,9 +7060,9 @@
           <t>inv-06.string_current_6_a</t>
         </is>
       </c>
-      <c r="I163" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7099,9 +7099,9 @@
           <t>inv-06.string_current_7_a</t>
         </is>
       </c>
-      <c r="I164" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7138,9 +7138,9 @@
           <t>inv-06.string_current_8_a</t>
         </is>
       </c>
-      <c r="I165" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7177,9 +7177,9 @@
           <t>inv-06.string_current_9_a</t>
         </is>
       </c>
-      <c r="I166" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7216,9 +7216,9 @@
           <t>inv-06.string_current_10_a</t>
         </is>
       </c>
-      <c r="I167" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7255,9 +7255,9 @@
           <t>inv-06.string_current_11_a</t>
         </is>
       </c>
-      <c r="I168" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7294,9 +7294,9 @@
           <t>inv-06.string_current_12_a</t>
         </is>
       </c>
-      <c r="I169" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7333,9 +7333,9 @@
           <t>inv-06.string_current_13_a</t>
         </is>
       </c>
-      <c r="I170" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7372,9 +7372,9 @@
           <t>inv-06.string_current_14_a</t>
         </is>
       </c>
-      <c r="I171" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7411,9 +7411,9 @@
           <t>inv-06.string_current_15_a</t>
         </is>
       </c>
-      <c r="I172" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7450,9 +7450,9 @@
           <t>inv-06.string_current_16_a</t>
         </is>
       </c>
-      <c r="I173" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7489,9 +7489,9 @@
           <t>inv-06.string_current_17_a</t>
         </is>
       </c>
-      <c r="I174" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7528,9 +7528,9 @@
           <t>inv-06.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I175" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7567,9 +7567,9 @@
           <t>inv-07.ac_power_kw</t>
         </is>
       </c>
-      <c r="I176" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7606,9 +7606,9 @@
           <t>inv-07.current_l1_a</t>
         </is>
       </c>
-      <c r="I177" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7645,9 +7645,9 @@
           <t>inv-07.current_l2_a</t>
         </is>
       </c>
-      <c r="I178" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7684,9 +7684,9 @@
           <t>inv-07.current_l3_a</t>
         </is>
       </c>
-      <c r="I179" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7723,9 +7723,9 @@
           <t>inv-07.dc_power_kw</t>
         </is>
       </c>
-      <c r="I180" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7762,9 +7762,9 @@
           <t>inv-07.frequency_hz</t>
         </is>
       </c>
-      <c r="I181" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7801,9 +7801,9 @@
           <t>inv-07.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I182" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7840,9 +7840,9 @@
           <t>inv-07.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I183" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7879,9 +7879,9 @@
           <t>inv-07.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I184" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7918,9 +7918,9 @@
           <t>inv-07.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I185" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7953,9 +7953,9 @@
           <t>inv-07.comm_error</t>
         </is>
       </c>
-      <c r="I186" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -7992,9 +7992,9 @@
           <t>inv-07.string_current_1_a</t>
         </is>
       </c>
-      <c r="I187" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8031,9 +8031,9 @@
           <t>inv-07.string_current_2_a</t>
         </is>
       </c>
-      <c r="I188" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8070,9 +8070,9 @@
           <t>inv-07.string_current_3_a</t>
         </is>
       </c>
-      <c r="I189" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8109,9 +8109,9 @@
           <t>inv-07.string_current_4_a</t>
         </is>
       </c>
-      <c r="I190" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8148,9 +8148,9 @@
           <t>inv-07.string_current_5_a</t>
         </is>
       </c>
-      <c r="I191" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8187,9 +8187,9 @@
           <t>inv-07.string_current_6_a</t>
         </is>
       </c>
-      <c r="I192" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8226,9 +8226,9 @@
           <t>inv-07.string_current_7_a</t>
         </is>
       </c>
-      <c r="I193" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8265,9 +8265,9 @@
           <t>inv-07.string_current_8_a</t>
         </is>
       </c>
-      <c r="I194" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8304,9 +8304,9 @@
           <t>inv-07.string_current_9_a</t>
         </is>
       </c>
-      <c r="I195" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8343,9 +8343,9 @@
           <t>inv-07.string_current_10_a</t>
         </is>
       </c>
-      <c r="I196" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8382,9 +8382,9 @@
           <t>inv-07.string_current_11_a</t>
         </is>
       </c>
-      <c r="I197" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8421,9 +8421,9 @@
           <t>inv-07.string_current_12_a</t>
         </is>
       </c>
-      <c r="I198" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8460,9 +8460,9 @@
           <t>inv-07.string_current_13_a</t>
         </is>
       </c>
-      <c r="I199" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8499,9 +8499,9 @@
           <t>inv-07.string_current_14_a</t>
         </is>
       </c>
-      <c r="I200" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8538,9 +8538,9 @@
           <t>inv-07.string_current_15_a</t>
         </is>
       </c>
-      <c r="I201" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8577,9 +8577,9 @@
           <t>inv-07.string_current_16_a</t>
         </is>
       </c>
-      <c r="I202" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8616,9 +8616,9 @@
           <t>inv-07.string_current_17_a</t>
         </is>
       </c>
-      <c r="I203" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8655,9 +8655,9 @@
           <t>inv-07.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I204" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8694,9 +8694,9 @@
           <t>inv-08.ac_power_kw</t>
         </is>
       </c>
-      <c r="I205" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8733,9 +8733,9 @@
           <t>inv-08.current_l1_a</t>
         </is>
       </c>
-      <c r="I206" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8772,9 +8772,9 @@
           <t>inv-08.current_l2_a</t>
         </is>
       </c>
-      <c r="I207" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8811,9 +8811,9 @@
           <t>inv-08.current_l3_a</t>
         </is>
       </c>
-      <c r="I208" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8850,9 +8850,9 @@
           <t>inv-08.dc_power_kw</t>
         </is>
       </c>
-      <c r="I209" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8889,9 +8889,9 @@
           <t>inv-08.frequency_hz</t>
         </is>
       </c>
-      <c r="I210" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8928,9 +8928,9 @@
           <t>inv-08.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I211" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -8967,9 +8967,9 @@
           <t>inv-08.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I212" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9006,9 +9006,9 @@
           <t>inv-08.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I213" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9045,9 +9045,9 @@
           <t>inv-08.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I214" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9080,9 +9080,9 @@
           <t>inv-08.comm_error</t>
         </is>
       </c>
-      <c r="I215" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9119,9 +9119,9 @@
           <t>inv-08.string_current_1_a</t>
         </is>
       </c>
-      <c r="I216" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9158,9 +9158,9 @@
           <t>inv-08.string_current_2_a</t>
         </is>
       </c>
-      <c r="I217" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9197,9 +9197,9 @@
           <t>inv-08.string_current_3_a</t>
         </is>
       </c>
-      <c r="I218" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9236,9 +9236,9 @@
           <t>inv-08.string_current_4_a</t>
         </is>
       </c>
-      <c r="I219" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9275,9 +9275,9 @@
           <t>inv-08.string_current_5_a</t>
         </is>
       </c>
-      <c r="I220" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9314,9 +9314,9 @@
           <t>inv-08.string_current_6_a</t>
         </is>
       </c>
-      <c r="I221" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9353,9 +9353,9 @@
           <t>inv-08.string_current_7_a</t>
         </is>
       </c>
-      <c r="I222" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9392,9 +9392,9 @@
           <t>inv-08.string_current_8_a</t>
         </is>
       </c>
-      <c r="I223" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9431,9 +9431,9 @@
           <t>inv-08.string_current_9_a</t>
         </is>
       </c>
-      <c r="I224" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9470,9 +9470,9 @@
           <t>inv-08.string_current_10_a</t>
         </is>
       </c>
-      <c r="I225" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9509,9 +9509,9 @@
           <t>inv-08.string_current_11_a</t>
         </is>
       </c>
-      <c r="I226" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9548,9 +9548,9 @@
           <t>inv-08.string_current_12_a</t>
         </is>
       </c>
-      <c r="I227" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9587,9 +9587,9 @@
           <t>inv-08.string_current_13_a</t>
         </is>
       </c>
-      <c r="I228" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9626,9 +9626,9 @@
           <t>inv-08.string_current_14_a</t>
         </is>
       </c>
-      <c r="I229" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9665,9 +9665,9 @@
           <t>inv-08.string_current_15_a</t>
         </is>
       </c>
-      <c r="I230" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9704,9 +9704,9 @@
           <t>inv-08.string_current_16_a</t>
         </is>
       </c>
-      <c r="I231" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9743,9 +9743,9 @@
           <t>inv-08.string_current_17_a</t>
         </is>
       </c>
-      <c r="I232" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9782,9 +9782,9 @@
           <t>inv-08.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I233" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9821,9 +9821,9 @@
           <t>inv-09.ac_power_kw</t>
         </is>
       </c>
-      <c r="I234" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9860,9 +9860,9 @@
           <t>inv-09.current_l1_a</t>
         </is>
       </c>
-      <c r="I235" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9899,9 +9899,9 @@
           <t>inv-09.current_l2_a</t>
         </is>
       </c>
-      <c r="I236" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9938,9 +9938,9 @@
           <t>inv-09.current_l3_a</t>
         </is>
       </c>
-      <c r="I237" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -9977,9 +9977,9 @@
           <t>inv-09.dc_power_kw</t>
         </is>
       </c>
-      <c r="I238" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10016,9 +10016,9 @@
           <t>inv-09.frequency_hz</t>
         </is>
       </c>
-      <c r="I239" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10055,9 +10055,9 @@
           <t>inv-09.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I240" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10094,9 +10094,9 @@
           <t>inv-09.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I241" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10133,9 +10133,9 @@
           <t>inv-09.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I242" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10172,9 +10172,9 @@
           <t>inv-09.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I243" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10207,9 +10207,9 @@
           <t>inv-09.comm_error</t>
         </is>
       </c>
-      <c r="I244" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10246,9 +10246,9 @@
           <t>inv-09.string_current_1_a</t>
         </is>
       </c>
-      <c r="I245" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10285,9 +10285,9 @@
           <t>inv-09.string_current_2_a</t>
         </is>
       </c>
-      <c r="I246" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10324,9 +10324,9 @@
           <t>inv-09.string_current_3_a</t>
         </is>
       </c>
-      <c r="I247" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10363,9 +10363,9 @@
           <t>inv-09.string_current_4_a</t>
         </is>
       </c>
-      <c r="I248" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10402,9 +10402,9 @@
           <t>inv-09.string_current_5_a</t>
         </is>
       </c>
-      <c r="I249" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10441,9 +10441,9 @@
           <t>inv-09.string_current_6_a</t>
         </is>
       </c>
-      <c r="I250" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10480,9 +10480,9 @@
           <t>inv-09.string_current_7_a</t>
         </is>
       </c>
-      <c r="I251" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10519,9 +10519,9 @@
           <t>inv-09.string_current_8_a</t>
         </is>
       </c>
-      <c r="I252" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10558,9 +10558,9 @@
           <t>inv-09.string_current_9_a</t>
         </is>
       </c>
-      <c r="I253" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10597,9 +10597,9 @@
           <t>inv-09.string_current_10_a</t>
         </is>
       </c>
-      <c r="I254" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10636,9 +10636,9 @@
           <t>inv-09.string_current_11_a</t>
         </is>
       </c>
-      <c r="I255" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10675,9 +10675,9 @@
           <t>inv-09.string_current_12_a</t>
         </is>
       </c>
-      <c r="I256" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10714,9 +10714,9 @@
           <t>inv-09.string_current_13_a</t>
         </is>
       </c>
-      <c r="I257" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10753,9 +10753,9 @@
           <t>inv-09.string_current_14_a</t>
         </is>
       </c>
-      <c r="I258" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10792,9 +10792,9 @@
           <t>inv-09.string_current_15_a</t>
         </is>
       </c>
-      <c r="I259" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10831,9 +10831,9 @@
           <t>inv-09.string_current_16_a</t>
         </is>
       </c>
-      <c r="I260" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10870,9 +10870,9 @@
           <t>inv-09.string_current_17_a</t>
         </is>
       </c>
-      <c r="I261" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10909,9 +10909,9 @@
           <t>inv-09.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I262" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10948,9 +10948,9 @@
           <t>inv-10.ac_power_kw</t>
         </is>
       </c>
-      <c r="I263" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -10987,9 +10987,9 @@
           <t>inv-10.current_l1_a</t>
         </is>
       </c>
-      <c r="I264" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11026,9 +11026,9 @@
           <t>inv-10.current_l2_a</t>
         </is>
       </c>
-      <c r="I265" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11065,9 +11065,9 @@
           <t>inv-10.current_l3_a</t>
         </is>
       </c>
-      <c r="I266" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11104,9 +11104,9 @@
           <t>inv-10.dc_power_kw</t>
         </is>
       </c>
-      <c r="I267" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11143,9 +11143,9 @@
           <t>inv-10.frequency_hz</t>
         </is>
       </c>
-      <c r="I268" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11182,9 +11182,9 @@
           <t>inv-10.voltage_l1_v</t>
         </is>
       </c>
-      <c r="I269" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11221,9 +11221,9 @@
           <t>inv-10.voltage_l2_v</t>
         </is>
       </c>
-      <c r="I270" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11260,9 +11260,9 @@
           <t>inv-10.voltage_l3_v</t>
         </is>
       </c>
-      <c r="I271" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11299,9 +11299,9 @@
           <t>inv-10.energy_today_kwh</t>
         </is>
       </c>
-      <c r="I272" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11334,9 +11334,9 @@
           <t>inv-10.comm_error</t>
         </is>
       </c>
-      <c r="I273" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11373,9 +11373,9 @@
           <t>inv-10.string_current_1_a</t>
         </is>
       </c>
-      <c r="I274" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11412,9 +11412,9 @@
           <t>inv-10.string_current_2_a</t>
         </is>
       </c>
-      <c r="I275" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11451,9 +11451,9 @@
           <t>inv-10.string_current_3_a</t>
         </is>
       </c>
-      <c r="I276" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11490,9 +11490,9 @@
           <t>inv-10.string_current_4_a</t>
         </is>
       </c>
-      <c r="I277" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11529,9 +11529,9 @@
           <t>inv-10.string_current_5_a</t>
         </is>
       </c>
-      <c r="I278" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11568,9 +11568,9 @@
           <t>inv-10.string_current_6_a</t>
         </is>
       </c>
-      <c r="I279" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11607,9 +11607,9 @@
           <t>inv-10.string_current_7_a</t>
         </is>
       </c>
-      <c r="I280" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11646,9 +11646,9 @@
           <t>inv-10.string_current_8_a</t>
         </is>
       </c>
-      <c r="I281" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11685,9 +11685,9 @@
           <t>inv-10.string_current_9_a</t>
         </is>
       </c>
-      <c r="I282" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11724,9 +11724,9 @@
           <t>inv-10.string_current_10_a</t>
         </is>
       </c>
-      <c r="I283" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11763,9 +11763,9 @@
           <t>inv-10.string_current_11_a</t>
         </is>
       </c>
-      <c r="I284" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11802,9 +11802,9 @@
           <t>inv-10.string_current_12_a</t>
         </is>
       </c>
-      <c r="I285" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11841,9 +11841,9 @@
           <t>inv-10.string_current_13_a</t>
         </is>
       </c>
-      <c r="I286" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11880,9 +11880,9 @@
           <t>inv-10.string_current_14_a</t>
         </is>
       </c>
-      <c r="I287" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11919,9 +11919,9 @@
           <t>inv-10.string_current_15_a</t>
         </is>
       </c>
-      <c r="I288" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11958,9 +11958,9 @@
           <t>inv-10.string_current_16_a</t>
         </is>
       </c>
-      <c r="I289" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -11997,9 +11997,9 @@
           <t>inv-10.string_current_17_a</t>
         </is>
       </c>
-      <c r="I290" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>
@@ -12036,9 +12036,9 @@
           <t>inv-10.energy_total_kwh</t>
         </is>
       </c>
-      <c r="I291" s="3" t="inlineStr">
-        <is>
-          <t>Pending commissioning</t>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
     </row>

</xml_diff>